<commit_message>
casi terminado campos corregidos
</commit_message>
<xml_diff>
--- a/plantillas/curriculum.xlsx
+++ b/plantillas/curriculum.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Isac\Documents\Formulario Servicio\formulario-servicio\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB892A40-7663-440B-B1D2-C7E73BC2F0C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEC6C0F9-42DC-4346-B93B-B4C7AE1F3FFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="715" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -367,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -390,17 +390,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -430,26 +424,23 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -462,15 +453,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -908,7 +890,7 @@
   <cols>
     <col min="1" max="1" width="39.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="23.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="39.140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="37.28515625" style="2" customWidth="1"/>
     <col min="5" max="5" width="21.7109375" style="2" customWidth="1"/>
     <col min="6" max="6" width="15.5703125" style="2" customWidth="1"/>
@@ -927,109 +909,109 @@
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
     </row>
     <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
     </row>
     <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="30"/>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
+      <c r="A5" s="27"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
     </row>
     <row r="6" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
     </row>
     <row r="7" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
     </row>
     <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
     </row>
     <row r="9" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
     </row>
     <row r="10" spans="1:7" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1059,12 +1041,12 @@
       <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="26"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="23"/>
     </row>
     <row r="14" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
@@ -1078,22 +1060,22 @@
       <c r="G14" s="4"/>
     </row>
     <row r="15" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
     </row>
     <row r="16" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="4"/>
-      <c r="C16" s="20"/>
+      <c r="C16" s="18"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
@@ -1104,7 +1086,7 @@
         <v>11</v>
       </c>
       <c r="B17" s="4"/>
-      <c r="C17" s="20"/>
+      <c r="C17" s="18"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
@@ -1114,58 +1096,56 @@
       <c r="A18" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
     </row>
     <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="17"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
     </row>
     <row r="20" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="33"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="34" t="s">
+      <c r="C21" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="34"/>
-      <c r="E21" s="13" t="s">
+      <c r="D21" s="11" t="s">
         <v>23</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="5"/>
+      <c r="A22" s="6"/>
       <c r="B22" s="6"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="11"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="1"/>
       <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
@@ -1173,45 +1153,45 @@
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
       <c r="E23" s="7"/>
-      <c r="F23" s="15"/>
+      <c r="F23" s="13"/>
       <c r="G23" s="7"/>
     </row>
     <row r="24" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="36" t="s">
+      <c r="A24" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="36"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
     </row>
     <row r="25" spans="1:7" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="37" t="s">
+      <c r="A25" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="39"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" ht="84" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
+    <row r="26" spans="1:7" ht="42" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="D26" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="12" t="s">
         <v>14</v>
       </c>
       <c r="F26" s="1"/>
@@ -1219,33 +1199,33 @@
     </row>
     <row r="27" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="11"/>
-      <c r="G27" s="9"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="20"/>
+      <c r="G27" s="8"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="33" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" x14ac:dyDescent="0.25"/>
+    <row r="34" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="49" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="50" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="51" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1431,12 +1411,10 @@
     <row r="231" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="232" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
+  <mergeCells count="13">
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A20:D20"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A4:G4"/>

</xml_diff>

<commit_message>
Sistema terminado (fin servicio social)
</commit_message>
<xml_diff>
--- a/plantillas/curriculum.xlsx
+++ b/plantillas/curriculum.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Isac\Documents\Formulario Servicio\formulario-servicio\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEC6C0F9-42DC-4346-B93B-B4C7AE1F3FFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD60105-A3B7-4632-B610-9977AF66CFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="715" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="FORMATO CURRICULUM TRANSPARENCI" sheetId="10" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'FORMATO CURRICULUM TRANSPARENCI'!$A$1:$G$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'FORMATO CURRICULUM TRANSPARENCI'!$A$1:$G$34</definedName>
   </definedNames>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>PODER JUDICIAL DEL ESTADO DE HIDALGO</t>
   </si>
@@ -97,9 +97,6 @@
     <t>DOCUMENTO QUE LO ACREDITA</t>
   </si>
   <si>
-    <t>(INCLUYENDO CARGOS DENTRO DEL PODER JUDICIAL ADMINISTRATIVOS O DE CARRERA JUDICIAL)</t>
-  </si>
-  <si>
     <t>NOMBRE DE LA LICENCIATURA, MAESTRIA, DOCTORADO O ESPECIALIDAD</t>
   </si>
   <si>
@@ -118,29 +115,17 @@
     <t>CURRICULUM VITAE</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">CARGO O PUESTO DESEMPEÑADO </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(REDACTADO CON PERSPECTIVA DE GÉNERO)</t>
-    </r>
-  </si>
-  <si>
     <t>LICENCIATURA</t>
+  </si>
+  <si>
+    <t>CARGO O PUESTO DESEMPEÑADO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,21 +162,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="15"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF7030A0"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -250,7 +220,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -332,42 +302,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -399,16 +338,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -427,6 +366,24 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -436,35 +393,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -909,68 +839,68 @@
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
     </row>
     <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
     </row>
     <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
+      <c r="A5" s="25"/>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
     </row>
     <row r="6" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
+      <c r="A6" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
     </row>
     <row r="7" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
     </row>
     <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
@@ -982,22 +912,22 @@
       <c r="G8" s="10"/>
     </row>
     <row r="9" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
     </row>
     <row r="10" spans="1:7" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>16</v>
@@ -1019,34 +949,34 @@
       <c r="A11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="23"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="29"/>
     </row>
     <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="21"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="23"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="29"/>
     </row>
     <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="23"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="29"/>
     </row>
     <row r="14" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
@@ -1061,7 +991,7 @@
     </row>
     <row r="15" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -1113,12 +1043,12 @@
       <c r="G19" s="15"/>
     </row>
     <row r="20" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
       <c r="E20"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
@@ -1131,7 +1061,7 @@
         <v>22</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>23</v>
@@ -1157,61 +1087,51 @@
       <c r="G23" s="7"/>
     </row>
     <row r="24" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="30" t="s">
+      <c r="A24" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="30"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:7" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="33"/>
+    <row r="25" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>14</v>
+      </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" ht="42" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-    </row>
-    <row r="27" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="20"/>
-      <c r="G27" s="8"/>
-    </row>
+    <row r="26" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="6"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="20"/>
+      <c r="G26" s="8"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="33" x14ac:dyDescent="0.25"/>
-    <row r="34" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="36" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1411,9 +1331,8 @@
     <row r="231" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="232" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="12">
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A25:E25"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>

</xml_diff>